<commit_message>
fix(pricing): 最低起步价23.90→28.90 + 年终结算minFee地板规则
- constants.js: 全部8种材料 minFee €23.90 → €28.90
- calcSettlement 重写: 传入minFee参数
  - 实际kg×费率 < 起步价 → 不予退款(已付最低起步价)
  - 实际kg×费率 ≥ 起步价 → 按合同§5(3)惩罚规则结算
  - actualFee永不低

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/回收费价目单_2026.xlsx
+++ b/projects/回收费价目单_2026.xlsx
@@ -1797,7 +1797,7 @@
         <v>16</v>
       </c>
       <c r="E5" s="24">
-        <v>23.9</v>
+        <v>28.9</v>
       </c>
       <c r="F5" s="25">
         <v>0</v>
@@ -1820,7 +1820,7 @@
         <v>16</v>
       </c>
       <c r="E6" s="31">
-        <v>23.9</v>
+        <v>28.9</v>
       </c>
       <c r="F6" s="32">
         <v>50</v>
@@ -1843,7 +1843,7 @@
         <v>16</v>
       </c>
       <c r="E7" s="38">
-        <v>23.9</v>
+        <v>28.9</v>
       </c>
       <c r="F7" s="39">
         <v>100</v>
@@ -1866,7 +1866,7 @@
         <v>17</v>
       </c>
       <c r="E8" s="45">
-        <v>23.9</v>
+        <v>28.9</v>
       </c>
       <c r="F8" s="46">
         <v>0</v>
@@ -1889,7 +1889,7 @@
         <v>17</v>
       </c>
       <c r="E9" s="45">
-        <v>23.9</v>
+        <v>28.9</v>
       </c>
       <c r="F9" s="46">
         <v>50</v>
@@ -1912,7 +1912,7 @@
         <v>17</v>
       </c>
       <c r="E10" s="45">
-        <v>23.9</v>
+        <v>28.9</v>
       </c>
       <c r="F10" s="46">
         <v>100</v>
@@ -1935,7 +1935,7 @@
         <v>17</v>
       </c>
       <c r="E11" s="45">
-        <v>23.9</v>
+        <v>28.9</v>
       </c>
       <c r="F11" s="46">
         <v>1000</v>
@@ -1958,7 +1958,7 @@
         <v>19</v>
       </c>
       <c r="E12" s="52">
-        <v>23.9</v>
+        <v>28.9</v>
       </c>
       <c r="F12" s="53">
         <v>0</v>
@@ -1981,7 +1981,7 @@
         <v>20</v>
       </c>
       <c r="E13" s="45">
-        <v>23.9</v>
+        <v>28.9</v>
       </c>
       <c r="F13" s="46">
         <v>0</v>
@@ -2004,7 +2004,7 @@
         <v>21</v>
       </c>
       <c r="E14" s="52">
-        <v>23.9</v>
+        <v>28.9</v>
       </c>
       <c r="F14" s="53">
         <v>0</v>
@@ -2027,7 +2027,7 @@
         <v>22</v>
       </c>
       <c r="E15" s="45">
-        <v>23.9</v>
+        <v>28.9</v>
       </c>
       <c r="F15" s="46">
         <v>0</v>
@@ -2050,7 +2050,7 @@
         <v>23</v>
       </c>
       <c r="E16" s="45">
-        <v>23.9</v>
+        <v>28.9</v>
       </c>
       <c r="F16" s="46">
         <v>0</v>
@@ -2073,7 +2073,7 @@
         <v>24</v>
       </c>
       <c r="E17" s="45">
-        <v>23.9</v>
+        <v>28.9</v>
       </c>
       <c r="F17" s="46">
         <v>0</v>
@@ -2096,7 +2096,7 @@
         <v>24</v>
       </c>
       <c r="E18" s="45">
-        <v>23.9</v>
+        <v>28.9</v>
       </c>
       <c r="F18" s="46">
         <v>100</v>
@@ -2119,7 +2119,7 @@
         <v>24</v>
       </c>
       <c r="E19" s="62">
-        <v>23.9</v>
+        <v>28.9</v>
       </c>
       <c r="F19" s="63">
         <v>200</v>

</xml_diff>